<commit_message>
Add module migration sunset backlog
</commit_message>
<xml_diff>
--- a/reports/module-data-integration-audit/2026-07-27/CURRENT_MODULE_DATA_INVENTORY.xlsx
+++ b/reports/module-data-integration-audit/2026-07-27/CURRENT_MODULE_DATA_INVENTORY.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="1" r:id="R72a70fd0161240ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inventory" sheetId="1" r:id="R6f846340a2db41f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7813,7 +7813,7 @@
         <x:v>Static repo audit only: requires live row profiling for nulls, duplicates, stale rows, broken links</x:v>
       </x:c>
       <x:c r="N104" s="5" t="str">
-        <x:v>scripts/qa/home-know-data-gate.mjs; src/lib/tower/tower-budget-rollups.ts; src/lib/tower/tower-semantic-projection.ts</x:v>
+        <x:v>scripts/audit/build-module-migration-sunset-backlog.mjs; scripts/qa/home-know-data-gate.mjs; src/lib/tower/tower-budget-rollups.ts; src/lib/tower/tower-semantic-projection.ts</x:v>
       </x:c>
       <x:c r="O104" s="5" t="str"/>
       <x:c r="P104" s="5" t="str">
@@ -7838,7 +7838,7 @@
         <x:v>id; client_id; tenant_key; canonical_record_id; record_type; record_subtype; title; source_id; source_file_id; source_system; source_record_id; source_file; source_sheet; source_row_number; owner; steward_owner; last_synced_at; last_validated_at; confidence; freshness_status; evidence_pointer; lifecycle_state; superseded_by_record_id; payload_hash</x:v>
       </x:c>
       <x:c r="W104" s="5" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="X104" s="5" t="str">
         <x:v>high: migration DDL parsed</x:v>

</xml_diff>